<commit_message>
Se agrego el login entre multiples usuarios con archivos separados para cada uno
</commit_message>
<xml_diff>
--- a/Reporte-EasyFinance-briamm.xlsx
+++ b/Reporte-EasyFinance-briamm.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -25,13 +25,22 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="0081c9fa"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -46,8 +55,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -413,31 +425,31 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E3"/>
+  <dimension ref="A1:E4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Fecha</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Producto</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Precio</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Cantidad</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Tipo</t>
         </is>
@@ -446,7 +458,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026/07/30</t>
+          <t>2026/07/31</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -455,10 +467,10 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>3.99</v>
+        <v>24</v>
       </c>
       <c r="D2" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
@@ -469,23 +481,46 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026/07/30</t>
+          <t>2026/07/31</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Colas</t>
+          <t>envios</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>3.99</v>
+        <v>24</v>
       </c>
       <c r="D3" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>+(Ingreso)</t>
+          <t>-(Egreso)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026/07/31</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>productos</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>24.04</v>
+      </c>
+      <c r="D4" t="n">
+        <v>3</v>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>-(Envío)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Se empezo a trabajar en la pantalla principal
</commit_message>
<xml_diff>
--- a/Reporte-EasyFinance-briamm.xlsx
+++ b/Reporte-EasyFinance-briamm.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E4"/>
+  <dimension ref="A1:E6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -521,6 +521,52 @@
       <c r="E4" t="inlineStr">
         <is>
           <t>-(Envío)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026/08/02</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>hojas blancas</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>3.99</v>
+      </c>
+      <c r="D5" t="n">
+        <v>8</v>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>+(Ingreso)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026/08/02</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>palos</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>7.99</v>
+      </c>
+      <c r="D6" t="n">
+        <v>5</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>-(Egreso)</t>
         </is>
       </c>
     </row>

</xml_diff>